<commit_message>
Agregar galería de fotos por producto, datos del comprador en checkout y mejoras de rendimiento
- Nueva hoja 'Imagenes' (producto_id, orden, url) para varias fotos por referencia,
  con galería de miniaturas en la ficha de producto (GaleriaProducto.jsx)
- Formulario obligatorio de nombre/teléfono/correo antes de enviar el pedido por
  WhatsApp, con validación e info incluida en el mensaje
- Catálogo con paginación ('Cargar más') en vez de renderizar todo de una vez
- Fotos con loading=lazy y resolución reducida en las tarjetas del catálogo
- Caché de 5 min en el Apps Script (CacheService) para sostener varias visitas
  concurrentes sin releer todo el Sheet en cada request
- Instructivo técnico y Excel base actualizados con la nueva hoja Imagenes
</commit_message>
<xml_diff>
--- a/docs/TezCanela_Inventario_Base.xlsx
+++ b/docs/TezCanela_Inventario_Base.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Léeme" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Productos" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Variantes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Imagenes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -484,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -504,6 +505,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -528,89 +530,106 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
+          <t>•  Pestaña "Imagenes": una fila por cada foto de un producto (con modelo, sin modelo, detalle, etc).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
           <t>•  Esta pestaña "Léeme" es solo informativa — no la lee el sitio web.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Los datos que ya están cargados son de EJEMPLO</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Las filas que ves en Productos y Variantes son productos ficticios, solo para que el formato</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>quede claro. Bórralas y reemplázalas por el inventario real cuando esté listo — o consulta el</t>
+          <t>Las filas que ves en Productos y Variantes son productos ficticios, solo para que el formato</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
+          <t>quede claro. Bórralas y reemplázalas por el inventario real cuando esté listo — o consulta el</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
           <t>manual "MANUAL_INVENTARIO.docx" para el paso a paso de cómo agregar/editar productos.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Reglas importantes</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>•  No cambiar los nombres de las pestañas ni de las columnas (fila 1 de cada pestaña).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>•  El "id" de Productos y el "producto_id" de Variantes deben coincidir exactamente.</t>
+          <t>•  No cambiar los nombres de las pestañas ni de las columnas (fila 1 de cada pestaña).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>•  No repetir el mismo "id" en dos productos distintos.</t>
+          <t>•  El "id" de Productos y el "producto_id" de Variantes deben coincidir exactamente.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>•  "precio" y "stock" van solo en números, sin puntos ni símbolos ($).</t>
+          <t>•  No repetir el mismo "id" en dos productos distintos.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
+          <t>•  "precio" y "stock" van solo en números, sin puntos ni símbolos ($).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
           <t>•  "activo" en VERDADERO muestra el producto en el catálogo; en FALSO lo oculta sin borrarlo.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>•  En "Imagenes", el "producto_id" debe coincidir con el "id" de Productos; "orden" 1 = portada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Este archivo se importó desde un Excel armado por JCS Emprende. Una vez esté en Google</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Sheets, hay que copiar la URL del Sheet y seguir docs/INSTRUCTIVO_TECNICO.md para publicarlo.</t>
         </is>
@@ -3209,4 +3228,70 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>producto_id</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>orden</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>p1</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/thumbnail?id=ID_DE_LA_FOTO_1&amp;sz=w1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>p1</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/thumbnail?id=ID_DE_LA_FOTO_2&amp;sz=w1000</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>